<commit_message>
formatted the generated attandance report
</commit_message>
<xml_diff>
--- a/backend/attendance_sheet/AIML_B,2023-27,DBMS (PCCCS501)_Register.xlsx
+++ b/backend/attendance_sheet/AIML_B,2023-27,DBMS (PCCCS501)_Register.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,8 +77,14 @@
       <color rgb="009CA3AF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -135,6 +141,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="004338CA"/>
         <bgColor rgb="004338CA"/>
       </patternFill>
@@ -186,7 +198,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -223,15 +235,20 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -603,7 +620,7 @@
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
     <col width="35" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
@@ -814,14 +831,14 @@
         </is>
       </c>
       <c r="D10" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="11" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -897,12 +914,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:R12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
@@ -918,9 +935,6 @@
     <col width="16" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -946,10 +960,6 @@
       <c r="P1" s="2" t="n"/>
       <c r="Q1" s="2" t="n"/>
       <c r="R1" s="2" t="n"/>
-      <c r="S1" s="2" t="n"/>
-      <c r="T1" s="2" t="n"/>
-      <c r="U1" s="2" t="n"/>
-      <c r="V1" s="2" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="n"/>
@@ -970,10 +980,6 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="n"/>
-      <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
-      <c r="U2" s="2" t="n"/>
-      <c r="V2" s="2" t="n"/>
     </row>
     <row r="3" ht="4" customHeight="1">
       <c r="A3" s="3" t="n"/>
@@ -994,10 +1000,6 @@
       <c r="P3" s="3" t="n"/>
       <c r="Q3" s="3" t="n"/>
       <c r="R3" s="3" t="n"/>
-      <c r="S3" s="3" t="n"/>
-      <c r="T3" s="3" t="n"/>
-      <c r="U3" s="3" t="n"/>
-      <c r="V3" s="3" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -1010,30 +1012,26 @@
           <t>PCCCS501</t>
         </is>
       </c>
-      <c r="G4" s="14" t="n"/>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>DEPARTMENT :</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>AIML</t>
         </is>
       </c>
-      <c r="N4" s="14" t="n"/>
-      <c r="O4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>SECTION :</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="P4" s="5" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="U4" s="14" t="n"/>
-      <c r="V4" s="14" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -1046,30 +1044,26 @@
           <t>5th</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n"/>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>YEAR :</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>3rd</t>
         </is>
       </c>
-      <c r="N5" s="14" t="n"/>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>ACADEMIC SESSION :</t>
         </is>
       </c>
-      <c r="R5" s="5" t="inlineStr">
+      <c r="P5" s="5" t="inlineStr">
         <is>
           <t>2023-27</t>
         </is>
       </c>
-      <c r="U5" s="14" t="n"/>
-      <c r="V5" s="14" t="n"/>
     </row>
     <row r="6" ht="4" customHeight="1">
       <c r="A6" s="3" t="n"/>
@@ -1090,10 +1084,6 @@
       <c r="P6" s="3" t="n"/>
       <c r="Q6" s="3" t="n"/>
       <c r="R6" s="3" t="n"/>
-      <c r="S6" s="3" t="n"/>
-      <c r="T6" s="3" t="n"/>
-      <c r="U6" s="3" t="n"/>
-      <c r="V6" s="3" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="15" t="inlineStr">
@@ -1186,21 +1176,6 @@
           <t>Percentage (in this month)</t>
         </is>
       </c>
-      <c r="S7" s="16" t="inlineStr">
-        <is>
-          <t>Total Present (throughout Session)</t>
-        </is>
-      </c>
-      <c r="T7" s="16" t="inlineStr">
-        <is>
-          <t>Total Absent (throughout Session)</t>
-        </is>
-      </c>
-      <c r="U7" s="16" t="inlineStr">
-        <is>
-          <t>Percentage (throughout Session)</t>
-        </is>
-      </c>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -1289,17 +1264,6 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="S8" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="U8" s="11" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
@@ -1388,17 +1352,6 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="S9" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T9" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="U9" s="11" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -1471,31 +1424,21 @@
           <t>–</t>
         </is>
       </c>
-      <c r="O10" s="11" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="O10" s="18" t="inlineStr">
+        <is>
+          <t>P
+06:19 PM</t>
         </is>
       </c>
       <c r="P10" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="Q10" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="R10" s="11" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="S10" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T10" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="U10" s="11" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+      <c r="R10" s="14" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -1586,17 +1529,6 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="S11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="U11" s="11" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
@@ -1685,35 +1617,24 @@
           <t>0.0%</t>
         </is>
       </c>
-      <c r="S12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="U12" s="11" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="O5:Q5"/>
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="J5:L5"/>
     <mergeCell ref="D5:F5"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="K4:M4"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="O4:Q4"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="P5:R5"/>
     <mergeCell ref="D4:F4"/>
-    <mergeCell ref="A1:V2"/>
-    <mergeCell ref="H4:J4"/>
-    <mergeCell ref="R4:T4"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="R5:T5"/>
-    <mergeCell ref="A6:V6"/>
-    <mergeCell ref="A3:V3"/>
+    <mergeCell ref="M4:O4"/>
+    <mergeCell ref="M5:O5"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="A1:R2"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="P4:R4"/>
+    <mergeCell ref="A6:R6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>